<commit_message>
Several bug fixes; modified step function arguments to avoid passing Step class to functions (to improve ability to use functions as API)
</commit_message>
<xml_diff>
--- a/ValidationTests.xlsx
+++ b/ValidationTests.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22527"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\Mac\Home\OneDrive - DataSoar\Projects\Excel_Steps\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{345C970D-6AF2-45D6-A85D-949D6CA31C12}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CB710A9-E12F-408B-A463-2C202774F28D}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-31073" yWindow="2130" windowWidth="21390" windowHeight="11917" firstSheet="1" activeTab="1" xr2:uid="{9DD4A102-5F6B-46DA-8541-48C3A19AE79F}"/>
+    <workbookView xWindow="1103" yWindow="1418" windowWidth="25312" windowHeight="15382" activeTab="2" xr2:uid="{9DD4A102-5F6B-46DA-8541-48C3A19AE79F}"/>
   </bookViews>
   <sheets>
     <sheet name="Lists" sheetId="2" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="Data" sheetId="587" r:id="rId3"/>
     <sheet name="Original Data" sheetId="585" r:id="rId4"/>
     <sheet name="ExcelSteps" sheetId="4" r:id="rId5"/>
+    <sheet name="XLStepsSettings" sheetId="588" state="veryHidden" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="List_Desc3">Lists!$A$2:$A$4</definedName>
@@ -30,7 +31,9 @@
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -38,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="84">
   <si>
     <t>Sheet</t>
   </si>
@@ -169,9 +172,6 @@
     <t>Calc_4</t>
   </si>
   <si>
-    <t>=Data_Data_1*Data_Data_2</t>
-  </si>
-  <si>
     <t>Calc_5</t>
   </si>
   <si>
@@ -250,16 +250,49 @@
     <t>Part B</t>
   </si>
   <si>
-    <t>=(Data_Data_1*Data_Data_2))</t>
-  </si>
-  <si>
     <t>Excel formula error</t>
   </si>
   <si>
-    <t>Individually enable rows 13-26 as shown by entering "Data" in Columm A and refreshing the table again</t>
-  </si>
-  <si>
     <t>All Row 13-26 validation cases should produce a Refresh Error dialog box as shown and should label the Column C cell with a comment as shown</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>txtval</t>
+  </si>
+  <si>
+    <t>boolean1</t>
+  </si>
+  <si>
+    <t>boolean2</t>
+  </si>
+  <si>
+    <t>ShtNameFrm</t>
+  </si>
+  <si>
+    <t>Instructions</t>
+  </si>
+  <si>
+    <t>Original Data</t>
+  </si>
+  <si>
+    <t>cBoxAppShtName</t>
+  </si>
+  <si>
+    <t>Data_t</t>
+  </si>
+  <si>
+    <t>=@Data_Data_1*@Data_Data_2</t>
+  </si>
+  <si>
+    <t>=(@Data_Data_1*@Data_Data_2))</t>
+  </si>
+  <si>
+    <t>Missing Step name</t>
+  </si>
+  <si>
+    <t>Individually enable rows 13-27 as shown by entering "Data" in Columm A and refreshing the table again</t>
   </si>
 </sst>
 </file>
@@ -1060,43 +1093,43 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="B2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="C3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="32" spans="3:3" x14ac:dyDescent="0.45">
       <c r="C32" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="33" spans="2:3" x14ac:dyDescent="0.45">
       <c r="C33" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="47" spans="2:3" x14ac:dyDescent="0.45">
       <c r="B47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C47" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
     </row>
     <row r="48" spans="2:3" x14ac:dyDescent="0.45">
       <c r="C48" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -1165,7 +1198,7 @@
         <v>23</v>
       </c>
       <c r="B3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C3" t="s">
         <v>37</v>
@@ -1310,7 +1343,7 @@
         <v>23</v>
       </c>
       <c r="B3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C3" t="s">
         <v>37</v>
@@ -1404,7 +1437,7 @@
     <col min="1" max="1" width="10" style="12" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="6.73046875" style="12" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13.3984375" style="13" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="25.9296875" style="14" customWidth="1"/>
+    <col min="4" max="4" width="31.796875" style="14" customWidth="1"/>
     <col min="5" max="5" width="10.06640625" style="12" customWidth="1"/>
     <col min="6" max="6" width="14.265625" style="12" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="31.9296875" style="15" customWidth="1"/>
@@ -1541,7 +1574,7 @@
         <v>8</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>43</v>
+        <v>80</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>22</v>
@@ -1559,13 +1592,13 @@
         <v>16</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>8</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>43</v>
+        <v>80</v>
       </c>
       <c r="E7" s="7" t="s">
         <v>42</v>
@@ -1583,22 +1616,22 @@
         <v>16</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>8</v>
       </c>
       <c r="D8" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="E8" s="7" t="s">
         <v>43</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>44</v>
       </c>
       <c r="F8" s="2" t="b">
         <v>1</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H8" s="2" t="s">
         <v>13</v>
@@ -1636,7 +1669,7 @@
       </c>
       <c r="B10" s="7"/>
       <c r="C10" s="5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D10" s="9" t="s">
         <v>17</v>
@@ -1656,7 +1689,7 @@
         <v>17</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D11" s="9"/>
       <c r="E11" s="7"/>
@@ -1694,7 +1727,7 @@
       <c r="E13" s="2"/>
       <c r="F13" s="2"/>
       <c r="G13" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H13" s="2"/>
       <c r="I13" s="2">
@@ -1713,7 +1746,7 @@
       <c r="E14" s="2"/>
       <c r="F14" s="2"/>
       <c r="G14" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H14" s="2"/>
       <c r="I14" s="2">
@@ -1734,7 +1767,7 @@
       <c r="E15" s="2"/>
       <c r="F15" s="2"/>
       <c r="G15" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="H15" s="2"/>
       <c r="I15" s="2"/>
@@ -1753,7 +1786,7 @@
       <c r="E16" s="2"/>
       <c r="F16" s="2"/>
       <c r="G16" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="H16" s="2"/>
       <c r="I16" s="2"/>
@@ -1772,7 +1805,7 @@
       <c r="E17" s="2"/>
       <c r="F17" s="2"/>
       <c r="G17" s="6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H17" s="2"/>
       <c r="I17" s="2" t="s">
@@ -1790,11 +1823,11 @@
         <v>10</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F18" s="2"/>
       <c r="G18" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H18" s="2"/>
       <c r="I18" s="2"/>
@@ -1814,7 +1847,7 @@
       <c r="E19" s="7"/>
       <c r="F19" s="2"/>
       <c r="G19" s="6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H19" s="2"/>
       <c r="I19" s="2"/>
@@ -1823,7 +1856,7 @@
     <row r="20" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A20" s="7"/>
       <c r="B20" s="7" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C20" s="5" t="s">
         <v>12</v>
@@ -1836,7 +1869,7 @@
       </c>
       <c r="F20" s="2"/>
       <c r="G20" s="6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H20" s="2"/>
       <c r="I20" s="2"/>
@@ -1858,7 +1891,7 @@
       </c>
       <c r="F21" s="2"/>
       <c r="G21" s="6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="H21" s="2"/>
       <c r="I21" s="2"/>
@@ -1881,13 +1914,13 @@
       <c r="A23" s="7"/>
       <c r="B23" s="7"/>
       <c r="C23" s="5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D23" s="9"/>
       <c r="E23" s="7"/>
       <c r="F23" s="2"/>
       <c r="G23" s="6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H23" s="2"/>
       <c r="I23" s="2"/>
@@ -1897,15 +1930,15 @@
       <c r="A24" s="7"/>
       <c r="B24" s="7"/>
       <c r="C24" s="5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E24" s="7"/>
       <c r="F24" s="2"/>
       <c r="G24" s="6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H24" s="2"/>
       <c r="I24" s="2"/>
@@ -1914,16 +1947,16 @@
     <row r="25" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A25" s="7"/>
       <c r="B25" s="7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D25" s="9"/>
       <c r="E25" s="7"/>
       <c r="F25" s="2"/>
       <c r="G25" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H25" s="2"/>
       <c r="I25" s="2"/>
@@ -1932,13 +1965,13 @@
     <row r="26" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A26" s="2"/>
       <c r="B26" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C26" s="5" t="s">
         <v>8</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>22</v>
@@ -1947,21 +1980,25 @@
         <v>1</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="H26" s="2"/>
       <c r="I26" s="2"/>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A27" s="2"/>
-      <c r="B27" s="2"/>
+      <c r="B27" s="2" t="s">
+        <v>17</v>
+      </c>
       <c r="C27" s="5"/>
       <c r="D27" s="4" t="s">
         <v>10</v>
       </c>
       <c r="E27" s="2"/>
       <c r="F27" s="2"/>
-      <c r="G27" s="6"/>
+      <c r="G27" s="6" t="s">
+        <v>82</v>
+      </c>
       <c r="H27" s="2"/>
       <c r="I27" s="2"/>
     </row>
@@ -2006,11 +2043,111 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C30" xr:uid="{9DC565B4-8D4C-4BCE-ACF2-20BB1ABACCCE}">
-      <formula1>"Col_Format, Col_Insert, Col_AddGroup, Col_Comment,Col_CondFormat, Col_Dropdown, Col_NumFormat, Col_Width, Tbl_Sort"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C30" xr:uid="{D80040AE-46D1-4EE6-8B5B-564647569365}">
+      <formula1>"Col_Format,Col_Insert,Col_AddGroup,Col_CondFormat,Col_Dropdown,Tbl_FreezeRow1,Tbl_Sort"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="0" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CAFA8E70-BE96-4022-BFCA-B74467D1C631}">
+  <sheetPr codeName="Sheet3"/>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C2" t="b">
+        <v>0</v>
+      </c>
+      <c r="D2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>75</v>
+      </c>
+      <c r="B3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" t="b">
+        <v>1</v>
+      </c>
+      <c r="D3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>75</v>
+      </c>
+      <c r="B4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C4" t="b">
+        <v>0</v>
+      </c>
+      <c r="D4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>75</v>
+      </c>
+      <c r="C5" t="b">
+        <v>0</v>
+      </c>
+      <c r="D5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>78</v>
+      </c>
+      <c r="C6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>75</v>
+      </c>
+      <c r="B7" t="s">
+        <v>79</v>
+      </c>
+      <c r="C7" t="b">
+        <v>0</v>
+      </c>
+      <c r="D7" t="b">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Start at Scenario Model validation
</commit_message>
<xml_diff>
--- a/ValidationTests.xlsx
+++ b/ValidationTests.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\Mac\Home\OneDrive - DataSoar\Projects\Excel_Steps\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{621628E9-AB98-4206-8454-664CA060C223}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C06E1FD-9D77-45FD-8FE3-BB0F11529AD1}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-22943" yWindow="2115" windowWidth="20161" windowHeight="12060" activeTab="3" xr2:uid="{9DD4A102-5F6B-46DA-8541-48C3A19AE79F}"/>
+    <workbookView xWindow="4133" yWindow="4035" windowWidth="20159" windowHeight="12060" activeTab="2" xr2:uid="{9DD4A102-5F6B-46DA-8541-48C3A19AE79F}"/>
   </bookViews>
   <sheets>
     <sheet name="Lists" sheetId="2" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="84">
   <si>
     <t>Data</t>
   </si>
@@ -290,6 +290,9 @@
   </si>
   <si>
     <t>Missing Step name</t>
+  </si>
+  <si>
+    <t>Data_t</t>
   </si>
 </sst>
 </file>
@@ -395,7 +398,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="1" applyFont="1"/>
@@ -419,6 +422,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Accent2" xfId="2" builtinId="33"/>
@@ -1562,11 +1566,11 @@
       <c r="C6" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="11" t="s">
         <v>58</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F6" s="5" t="b">
         <v>1</v>
@@ -2005,7 +2009,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CAFA8E70-BE96-4022-BFCA-B74467D1C631}">
   <sheetPr codeName="Sheet3"/>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.45">
@@ -2083,6 +2087,20 @@
         <v>1</v>
       </c>
     </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B7" t="s">
+        <v>83</v>
+      </c>
+      <c r="C7" t="b">
+        <v>0</v>
+      </c>
+      <c r="D7" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>